<commit_message>
Update ddPCR scatterplots and E200K outputs
</commit_message>
<xml_diff>
--- a/results/ddPCR/SNV_data_final.xlsx
+++ b/results/ddPCR/SNV_data_final.xlsx
@@ -5270,7 +5270,7 @@
         <v>0.00458655740654583</v>
       </c>
       <c r="L92" t="n">
-        <v>0.0649899108938712</v>
+        <v>0.0649899108938713</v>
       </c>
       <c r="M92" t="n">
         <v>15</v>
@@ -6814,7 +6814,7 @@
         <v>17378</v>
       </c>
       <c r="J123" t="n">
-        <v>49.8996043885338</v>
+        <v>49.8996043885337</v>
       </c>
       <c r="K123" t="n">
         <v>49.139483664773</v>
@@ -7414,13 +7414,13 @@
         <v>14951</v>
       </c>
       <c r="J135" t="n">
-        <v>0.00593709791742938</v>
+        <v>0.00592910048452141</v>
       </c>
       <c r="K135" t="n">
-        <v>0.00161730327749761</v>
+        <v>0.00161512325920015</v>
       </c>
       <c r="L135" t="n">
-        <v>0.0152140469181478</v>
+        <v>0.0151936037739392</v>
       </c>
       <c r="M135" t="n">
         <v>17</v>
@@ -7558,19 +7558,19 @@
         <v>0</v>
       </c>
       <c r="H138" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="I138" t="n">
         <v>16472</v>
       </c>
       <c r="J138" t="n">
-        <v>0.0164569280588581</v>
+        <v>0.0151674090614083</v>
       </c>
       <c r="K138" t="n">
-        <v>0.00875640873553979</v>
+        <v>0.00783197210892294</v>
       </c>
       <c r="L138" t="n">
-        <v>0.0281797678981566</v>
+        <v>0.0265292547864409</v>
       </c>
       <c r="M138" t="n">
         <v>18</v>
@@ -8008,19 +8008,19 @@
         <v>1</v>
       </c>
       <c r="H147" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="I147" t="n">
         <v>45458</v>
       </c>
       <c r="J147" t="n">
-        <v>0.0237803171174049</v>
+        <v>0.0225861970027339</v>
       </c>
       <c r="K147" t="n">
-        <v>0.0145252895048298</v>
+        <v>0.0135980573882371</v>
       </c>
       <c r="L147" t="n">
-        <v>0.0367288965082101</v>
+        <v>0.0352731471757438</v>
       </c>
       <c r="M147" t="n">
         <v>69</v>
@@ -8214,7 +8214,7 @@
         <v>28557</v>
       </c>
       <c r="J151" t="n">
-        <v>0.0712170185979904</v>
+        <v>0.0712170185979905</v>
       </c>
       <c r="K151" t="n">
         <v>0.0460894300139205</v>
@@ -8308,19 +8308,19 @@
         <v>1</v>
       </c>
       <c r="H153" t="n">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="I153" t="n">
         <v>43094</v>
       </c>
       <c r="J153" t="n">
-        <v>0.314507563935298</v>
+        <v>0.31366196417639</v>
       </c>
       <c r="K153" t="n">
-        <v>0.281988600584221</v>
+        <v>0.281184756947227</v>
       </c>
       <c r="L153" t="n">
-        <v>0.349772198537191</v>
+        <v>0.348885397284553</v>
       </c>
       <c r="M153" t="n">
         <v>66</v>
@@ -12867,7 +12867,7 @@
         <v>0.0281656435774004</v>
       </c>
       <c r="K244" t="n">
-        <v>0.0185576723626286</v>
+        <v>0.0185576723626285</v>
       </c>
       <c r="L244" t="n">
         <v>0.0409925348551718</v>
@@ -15317,10 +15317,10 @@
         <v>0.0200406285296919</v>
       </c>
       <c r="K293" t="n">
-        <v>0.00242723715163795</v>
+        <v>0.00242723715163796</v>
       </c>
       <c r="L293" t="n">
-        <v>0.0723854955259818</v>
+        <v>0.0723854955259819</v>
       </c>
       <c r="M293" t="n">
         <v>15</v>
@@ -16270,7 +16270,7 @@
         <v>0.00750427414216105</v>
       </c>
       <c r="L312" t="n">
-        <v>0.0705123253394388</v>
+        <v>0.0705123253394389</v>
       </c>
       <c r="M312" t="n">
         <v>13</v>
@@ -19317,7 +19317,7 @@
         <v>0.0200722200493538</v>
       </c>
       <c r="K373" t="n">
-        <v>0.0073657977981381</v>
+        <v>0.00736579779813811</v>
       </c>
       <c r="L373" t="n">
         <v>0.0436971452173887</v>
@@ -19417,7 +19417,7 @@
         <v>0.0215618065106053</v>
       </c>
       <c r="K375" t="n">
-        <v>0.00791229957544402</v>
+        <v>0.00791229957544404</v>
       </c>
       <c r="L375" t="n">
         <v>0.0469420772746819</v>
@@ -20314,13 +20314,13 @@
         <v>13593</v>
       </c>
       <c r="J393" t="n">
-        <v>0.016431396935137</v>
+        <v>0.0163826295301539</v>
       </c>
       <c r="K393" t="n">
-        <v>0.00847987815483543</v>
+        <v>0.00845458728775358</v>
       </c>
       <c r="L393" t="n">
-        <v>0.0287691407221729</v>
+        <v>0.0286844752161368</v>
       </c>
       <c r="M393" t="n">
         <v>15</v>
@@ -23317,7 +23317,7 @@
         <v>0.00790401994678377</v>
       </c>
       <c r="K453" t="n">
-        <v>0.000957207820179326</v>
+        <v>0.000957207820179324</v>
       </c>
       <c r="L453" t="n">
         <v>0.0285559013965602</v>
@@ -25708,19 +25708,19 @@
         <v>0</v>
       </c>
       <c r="H501" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I501" t="n">
         <v>11440</v>
       </c>
       <c r="J501" t="n">
-        <v>0.00611574355199338</v>
+        <v>0.00489244079125493</v>
       </c>
       <c r="K501" t="n">
-        <v>0.00198007847946259</v>
+        <v>0.00133003913336018</v>
       </c>
       <c r="L501" t="n">
-        <v>0.0143720210023291</v>
+        <v>0.0126088195435542</v>
       </c>
       <c r="M501" t="n">
         <v>13</v>
@@ -30664,13 +30664,13 @@
         <v>16833</v>
       </c>
       <c r="J600" t="n">
-        <v>0.0153811339451785</v>
+        <v>0.0153609369317713</v>
       </c>
       <c r="K600" t="n">
-        <v>0.00618346430474029</v>
+        <v>0.00617534288574729</v>
       </c>
       <c r="L600" t="n">
-        <v>0.0316992178963198</v>
+        <v>0.0316576161899308</v>
       </c>
       <c r="M600" t="n">
         <v>18</v>
@@ -32314,13 +32314,13 @@
         <v>30815</v>
       </c>
       <c r="J633" t="n">
-        <v>0.112548222194535</v>
+        <v>0.112514260776809</v>
       </c>
       <c r="K633" t="n">
-        <v>0.0897524921377716</v>
+        <v>0.0897253950989989</v>
       </c>
       <c r="L633" t="n">
-        <v>0.139383849879381</v>
+        <v>0.139341817843436</v>
       </c>
       <c r="M633" t="n">
         <v>37</v>
@@ -33017,7 +33017,7 @@
         <v>0.00428434157460931</v>
       </c>
       <c r="K647" t="n">
-        <v>0.000518817658943747</v>
+        <v>0.000518817658943746</v>
       </c>
       <c r="L647" t="n">
         <v>0.0154845381479274</v>

</xml_diff>

<commit_message>
Regenerate ddPCR outputs for corrected gates
</commit_message>
<xml_diff>
--- a/results/ddPCR/SNV_data_final.xlsx
+++ b/results/ddPCR/SNV_data_final.xlsx
@@ -9508,19 +9508,19 @@
         <v>0</v>
       </c>
       <c r="H177" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I177" t="n">
         <v>15056</v>
       </c>
       <c r="J177" t="n">
-        <v>0.0180140131218616</v>
+        <v>0.0140105291155955</v>
       </c>
       <c r="K177" t="n">
-        <v>0.00823544772020317</v>
+        <v>0.00563202260818086</v>
       </c>
       <c r="L177" t="n">
-        <v>0.0342129340852272</v>
+        <v>0.0288800348467268</v>
       </c>
       <c r="M177" t="n">
         <v>15</v>
@@ -9808,19 +9808,19 @@
         <v>0</v>
       </c>
       <c r="H183" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="I183" t="n">
         <v>15160</v>
       </c>
       <c r="J183" t="n">
-        <v>0.00386801771462629</v>
+        <v>0.00309433603066978</v>
       </c>
       <c r="K183" t="n">
-        <v>0.00124576515395246</v>
+        <v>0.000837757741890053</v>
       </c>
       <c r="L183" t="n">
-        <v>0.00915300220202122</v>
+        <v>0.00802668781386873</v>
       </c>
       <c r="M183" t="n">
         <v>15</v>
@@ -9958,19 +9958,19 @@
         <v>0</v>
       </c>
       <c r="H186" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="I186" t="n">
         <v>16723</v>
       </c>
       <c r="J186" t="n">
-        <v>0.0109416864386727</v>
+        <v>0.00683822107958527</v>
       </c>
       <c r="K186" t="n">
-        <v>0.00472218689205414</v>
+        <v>0.00221984952625984</v>
       </c>
       <c r="L186" t="n">
-        <v>0.0215777586995252</v>
+        <v>0.0159697890654529</v>
       </c>
       <c r="M186" t="n">
         <v>17</v>
@@ -10408,19 +10408,19 @@
         <v>0</v>
       </c>
       <c r="H195" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I195" t="n">
         <v>15775</v>
       </c>
       <c r="J195" t="n">
-        <v>0.00644195909236445</v>
+        <v>0.00536818668996907</v>
       </c>
       <c r="K195" t="n">
-        <v>0.00236206040287471</v>
+        <v>0.0017417916340444</v>
       </c>
       <c r="L195" t="n">
-        <v>0.0140533441454258</v>
+        <v>0.0125545264885204</v>
       </c>
       <c r="M195" t="n">
         <v>16</v>
@@ -10708,19 +10708,19 @@
         <v>0</v>
       </c>
       <c r="H201" t="n">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="I201" t="n">
         <v>16123</v>
       </c>
       <c r="J201" t="n">
-        <v>0.0138703454972834</v>
+        <v>0.0107877097144092</v>
       </c>
       <c r="K201" t="n">
-        <v>0.00634039185722858</v>
+        <v>0.00433611178850993</v>
       </c>
       <c r="L201" t="n">
-        <v>0.0263494343287488</v>
+        <v>0.0222417110583841</v>
       </c>
       <c r="M201" t="n">
         <v>16</v>
@@ -11008,19 +11008,19 @@
         <v>0</v>
       </c>
       <c r="H207" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I207" t="n">
         <v>17518</v>
       </c>
       <c r="J207" t="n">
-        <v>0.00286188336610586</v>
+        <v>0.00214636661013578</v>
       </c>
       <c r="K207" t="n">
-        <v>0.000777471556591257</v>
+        <v>0.000441723923556918</v>
       </c>
       <c r="L207" t="n">
-        <v>0.00738484101818401</v>
+        <v>0.00631801355512601</v>
       </c>
       <c r="M207" t="n">
         <v>17</v>
@@ -11458,19 +11458,19 @@
         <v>0</v>
       </c>
       <c r="H216" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I216" t="n">
         <v>16294</v>
       </c>
       <c r="J216" t="n">
-        <v>0.01164696004485</v>
+        <v>0.010093568928626</v>
       </c>
       <c r="K216" t="n">
-        <v>0.00645400111052113</v>
+        <v>0.00532643208135552</v>
       </c>
       <c r="L216" t="n">
-        <v>0.0194464336946081</v>
+        <v>0.0174619011630262</v>
       </c>
       <c r="M216" t="n">
         <v>16</v>
@@ -11758,19 +11758,19 @@
         <v>0</v>
       </c>
       <c r="H222" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="I222" t="n">
         <v>17828</v>
       </c>
       <c r="J222" t="n">
-        <v>0.00632864822240416</v>
+        <v>0.00361616416710011</v>
       </c>
       <c r="K222" t="n">
-        <v>0.00254166379703963</v>
+        <v>0.000984675377769694</v>
       </c>
       <c r="L222" t="n">
-        <v>0.0130733784213051</v>
+        <v>0.00927917197455792</v>
       </c>
       <c r="M222" t="n">
         <v>18</v>
@@ -11908,19 +11908,19 @@
         <v>0</v>
       </c>
       <c r="H225" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I225" t="n">
         <v>17488</v>
       </c>
       <c r="J225" t="n">
-        <v>0.00238130473304697</v>
+        <v>0.00158750369645045</v>
       </c>
       <c r="K225" t="n">
-        <v>0.000490590594308017</v>
+        <v>0.000192150039561377</v>
       </c>
       <c r="L225" t="n">
-        <v>0.00698832151815359</v>
+        <v>0.00575644720397774</v>
       </c>
       <c r="M225" t="n">
         <v>17</v>
@@ -12308,19 +12308,19 @@
         <v>0</v>
       </c>
       <c r="H233" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="I233" t="n">
         <v>15330</v>
       </c>
       <c r="J233" t="n">
-        <v>0.0244668432777965</v>
+        <v>0.0203579310343545</v>
       </c>
       <c r="K233" t="n">
-        <v>0.0126394000912042</v>
+        <v>0.00976042910112069</v>
       </c>
       <c r="L233" t="n">
-        <v>0.0427595849337368</v>
+        <v>0.0374562081793538</v>
       </c>
       <c r="M233" t="n">
         <v>15</v>
@@ -12414,13 +12414,13 @@
         <v>16937</v>
       </c>
       <c r="J235" t="n">
-        <v>0.00558923452787199</v>
+        <v>0.00557931678344893</v>
       </c>
       <c r="K235" t="n">
-        <v>0.00115257146152937</v>
+        <v>0.00115052601099749</v>
       </c>
       <c r="L235" t="n">
-        <v>0.0163387422632032</v>
+        <v>0.016309768184658</v>
       </c>
       <c r="M235" t="n">
         <v>17</v>
@@ -13664,13 +13664,13 @@
         <v>14770</v>
       </c>
       <c r="J260" t="n">
-        <v>0.010104659492478</v>
+        <v>0.0101330276124825</v>
       </c>
       <c r="K260" t="n">
-        <v>0.00370733550802742</v>
+        <v>0.00371775050353731</v>
       </c>
       <c r="L260" t="n">
-        <v>0.0220088761699113</v>
+        <v>0.0220705523385981</v>
       </c>
       <c r="M260" t="n">
         <v>21</v>
@@ -13964,13 +13964,13 @@
         <v>15018</v>
       </c>
       <c r="J266" t="n">
-        <v>0.00971476049210114</v>
+        <v>0.00971841999791206</v>
       </c>
       <c r="K266" t="n">
-        <v>0.00264679067514426</v>
+        <v>0.00264778787220649</v>
       </c>
       <c r="L266" t="n">
-        <v>0.0248799367989624</v>
+        <v>0.0248893039967551</v>
       </c>
       <c r="M266" t="n">
         <v>21</v>
@@ -14514,13 +14514,13 @@
         <v>15549</v>
       </c>
       <c r="J277" t="n">
-        <v>0.0264174201426192</v>
+        <v>0.0264228987202176</v>
       </c>
       <c r="K277" t="n">
-        <v>0.010621110056127</v>
+        <v>0.0106233130904565</v>
       </c>
       <c r="L277" t="n">
-        <v>0.0544348902415863</v>
+        <v>0.0544461756952827</v>
       </c>
       <c r="M277" t="n">
         <v>25</v>
@@ -15164,13 +15164,13 @@
         <v>23524</v>
       </c>
       <c r="J290" t="n">
-        <v>0.0121185532369918</v>
+        <v>0.0121202499026388</v>
       </c>
       <c r="K290" t="n">
-        <v>0.00393485490791686</v>
+        <v>0.00393540585928918</v>
       </c>
       <c r="L290" t="n">
-        <v>0.0282823475707711</v>
+        <v>0.0282863065095344</v>
       </c>
       <c r="M290" t="n">
         <v>31</v>
@@ -16370,7 +16370,7 @@
         <v>0</v>
       </c>
       <c r="L314" t="n">
-        <v>0.00398276305335548</v>
+        <v>0.00401294849471934</v>
       </c>
       <c r="M314" t="n">
         <v>22</v>
@@ -17158,19 +17158,19 @@
         <v>0</v>
       </c>
       <c r="H330" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I330" t="n">
         <v>16209</v>
       </c>
       <c r="J330" t="n">
-        <v>0.00148541725906939</v>
+        <v>0.000742691233945346</v>
       </c>
       <c r="K330" t="n">
-        <v>0.000179585180102617</v>
+        <v>0.0000187968917739303</v>
       </c>
       <c r="L330" t="n">
-        <v>0.00541368330659393</v>
+        <v>0.00417050781509146</v>
       </c>
       <c r="M330" t="n">
         <v>16</v>
@@ -17308,19 +17308,19 @@
         <v>0</v>
       </c>
       <c r="H333" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="I333" t="n">
         <v>15925</v>
       </c>
       <c r="J333" t="n">
-        <v>0.00259623425532269</v>
+        <v>0.00129805245430271</v>
       </c>
       <c r="K333" t="n">
-        <v>0.000689307526978192</v>
+        <v>0.000155664981042168</v>
       </c>
       <c r="L333" t="n">
-        <v>0.00682436201747195</v>
+        <v>0.00479400385863599</v>
       </c>
       <c r="M333" t="n">
         <v>16</v>
@@ -17758,19 +17758,19 @@
         <v>0</v>
       </c>
       <c r="H342" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="I342" t="n">
         <v>16877</v>
       </c>
       <c r="J342" t="n">
-        <v>0.00232247473681316</v>
+        <v>0.000774124358075731</v>
       </c>
       <c r="K342" t="n">
-        <v>0.000478198256287262</v>
+        <v>0.0000195956356421816</v>
       </c>
       <c r="L342" t="n">
-        <v>0.00682772868471219</v>
+        <v>0.00433375089711716</v>
       </c>
       <c r="M342" t="n">
         <v>17</v>
@@ -17914,13 +17914,13 @@
         <v>15897</v>
       </c>
       <c r="J345" t="n">
-        <v>0.00118307490208265</v>
+        <v>0.00118021087124745</v>
       </c>
       <c r="K345" t="n">
-        <v>0.0000299515088899638</v>
+        <v>0.0000298789936075782</v>
       </c>
       <c r="L345" t="n">
-        <v>0.00659826140969555</v>
+        <v>0.0065823451561835</v>
       </c>
       <c r="M345" t="n">
         <v>16</v>
@@ -22514,13 +22514,13 @@
         <v>24554</v>
       </c>
       <c r="J437" t="n">
-        <v>0.00583610303874001</v>
+        <v>0.00583749109460355</v>
       </c>
       <c r="K437" t="n">
-        <v>0.00159008269262548</v>
+        <v>0.00159046091568348</v>
       </c>
       <c r="L437" t="n">
-        <v>0.0149451436064332</v>
+        <v>0.0149486969544557</v>
       </c>
       <c r="M437" t="n">
         <v>32</v>

</xml_diff>

<commit_message>
Regenerate ddPCR outputs after quality-control update
</commit_message>
<xml_diff>
--- a/results/ddPCR/SNV_data_final.xlsx
+++ b/results/ddPCR/SNV_data_final.xlsx
@@ -4370,10 +4370,10 @@
         <v>0.0395112628427656</v>
       </c>
       <c r="M74" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="N74" t="n">
-        <v>0.122309197651663</v>
+        <v>0.220156555772994</v>
       </c>
       <c r="O74" t="b">
         <v>0</v>
@@ -4520,10 +4520,10 @@
         <v>0.0318750230176824</v>
       </c>
       <c r="M77" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="N77" t="n">
-        <v>0.118260869565217</v>
+        <v>0.215652173913043</v>
       </c>
       <c r="O77" t="b">
         <v>0</v>
@@ -4670,10 +4670,10 @@
         <v>0.0214716780735992</v>
       </c>
       <c r="M80" t="n">
-        <v>18</v>
+        <v>31</v>
       </c>
       <c r="N80" t="n">
-        <v>0.122766334742873</v>
+        <v>0.211430909834947</v>
       </c>
       <c r="O80" t="b">
         <v>0</v>
@@ -4820,10 +4820,10 @@
         <v>0.0396867753506377</v>
       </c>
       <c r="M83" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="N83" t="n">
-        <v>0.122438984572688</v>
+        <v>0.220390172230838</v>
       </c>
       <c r="O83" t="b">
         <v>0</v>
@@ -4970,10 +4970,10 @@
         <v>0.0474790543977189</v>
       </c>
       <c r="M86" t="n">
-        <v>17</v>
+        <v>31</v>
       </c>
       <c r="N86" t="n">
-        <v>0.117411423440845</v>
+        <v>0.214103183921542</v>
       </c>
       <c r="O86" t="b">
         <v>0</v>
@@ -5120,10 +5120,10 @@
         <v>0.117633304299542</v>
       </c>
       <c r="M89" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="N89" t="n">
-        <v>0.119579081632653</v>
+        <v>0.215242346938776</v>
       </c>
       <c r="O89" t="b">
         <v>0</v>
@@ -5270,10 +5270,10 @@
         <v>0.0198464966523898</v>
       </c>
       <c r="M92" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="N92" t="n">
-        <v>0.122425464496615</v>
+        <v>0.216044937346968</v>
       </c>
       <c r="O92" t="b">
         <v>0</v>
@@ -5420,10 +5420,10 @@
         <v>0.0649899108938713</v>
       </c>
       <c r="M95" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="N95" t="n">
-        <v>0.121911573472042</v>
+        <v>0.219440832249675</v>
       </c>
       <c r="O95" t="b">
         <v>0</v>
@@ -5570,10 +5570,10 @@
         <v>0.057776992013009</v>
       </c>
       <c r="M98" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="N98" t="n">
-        <v>0.121680624150025</v>
+        <v>0.214730513205927</v>
       </c>
       <c r="O98" t="b">
         <v>0</v>
@@ -5720,10 +5720,10 @@
         <v>0.0183983169247508</v>
       </c>
       <c r="M101" t="n">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="N101" t="n">
-        <v>0.126508369015181</v>
+        <v>0.223822499026859</v>
       </c>
       <c r="O101" t="b">
         <v>0</v>
@@ -5870,10 +5870,10 @@
         <v>0.0120817225587311</v>
       </c>
       <c r="M104" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="N104" t="n">
-        <v>0.125225013696486</v>
+        <v>0.21914377396885</v>
       </c>
       <c r="O104" t="b">
         <v>0</v>
@@ -12470,10 +12470,10 @@
         <v>0.0205912448556729</v>
       </c>
       <c r="M236" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="N236" t="n">
-        <v>0.122699386503067</v>
+        <v>0.0649584987369181</v>
       </c>
       <c r="O236" t="b">
         <v>0</v>
@@ -12520,10 +12520,10 @@
         <v>0.0285345552384346</v>
       </c>
       <c r="M237" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N237" t="n">
-        <v>0.0989201220014838</v>
+        <v>0.0659467480009892</v>
       </c>
       <c r="O237" t="b">
         <v>0</v>
@@ -12620,10 +12620,10 @@
         <v>0.0274987554911442</v>
       </c>
       <c r="M239" t="n">
-        <v>19</v>
+        <v>10</v>
       </c>
       <c r="N239" t="n">
-        <v>0.117975783918038</v>
+        <v>0.0620925178515989</v>
       </c>
       <c r="O239" t="b">
         <v>0</v>
@@ -12670,13 +12670,13 @@
         <v>0.0585564719758217</v>
       </c>
       <c r="M240" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N240" t="n">
-        <v>0.103775844176579</v>
+        <v>0.0718448151991698</v>
       </c>
       <c r="O240" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P240" t="b">
         <v>0</v>
@@ -12770,10 +12770,10 @@
         <v>0.0161459719868957</v>
       </c>
       <c r="M242" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="N242" t="n">
-        <v>0.122009082898394</v>
+        <v>0.0677828238324409</v>
       </c>
       <c r="O242" t="b">
         <v>0</v>
@@ -12820,10 +12820,10 @@
         <v>0.0181490643352089</v>
       </c>
       <c r="M243" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="N243" t="n">
-        <v>0.100050025012506</v>
+        <v>0.0643178732223254</v>
       </c>
       <c r="O243" t="b">
         <v>0</v>
@@ -12920,10 +12920,10 @@
         <v>0.0175636231781437</v>
       </c>
       <c r="M245" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="N245" t="n">
-        <v>0.117970900511207</v>
+        <v>0.0655393891728929</v>
       </c>
       <c r="O245" t="b">
         <v>0</v>
@@ -12970,10 +12970,10 @@
         <v>0.0157044971918804</v>
       </c>
       <c r="M246" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="N246" t="n">
-        <v>0.103542637378892</v>
+        <v>0.0665631240292878</v>
       </c>
       <c r="O246" t="b">
         <v>0</v>
@@ -13220,10 +13220,10 @@
         <v>0.112223546186696</v>
       </c>
       <c r="M251" t="n">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="N251" t="n">
-        <v>0.125740973594396</v>
+        <v>0.0718519849110832</v>
       </c>
       <c r="O251" t="b">
         <v>0</v>
@@ -13270,10 +13270,10 @@
         <v>0.0258888550888256</v>
       </c>
       <c r="M252" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="N252" t="n">
-        <v>0.109051254089422</v>
+        <v>0.0693962526023595</v>
       </c>
       <c r="O252" t="b">
         <v>0</v>
@@ -14120,10 +14120,10 @@
         <v>0.023170510100858</v>
       </c>
       <c r="M269" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="N269" t="n">
-        <v>0.119323366322735</v>
+        <v>0.0631711939355654</v>
       </c>
       <c r="O269" t="b">
         <v>0</v>
@@ -14170,10 +14170,10 @@
         <v>0.039475269172782</v>
       </c>
       <c r="M270" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N270" t="n">
-        <v>0.102467092299204</v>
+        <v>0.0709387562071412</v>
       </c>
       <c r="O270" t="b">
         <v>0</v>
@@ -14270,10 +14270,10 @@
         <v>0.0180421879892845</v>
       </c>
       <c r="M272" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N272" t="n">
-        <v>0.120404559319313</v>
+        <v>0.0642157649703002</v>
       </c>
       <c r="O272" t="b">
         <v>0</v>
@@ -14320,10 +14320,10 @@
         <v>0.0157835464883712</v>
       </c>
       <c r="M273" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N273" t="n">
-        <v>0.0987466767945309</v>
+        <v>0.0683630839346753</v>
       </c>
       <c r="O273" t="b">
         <v>0</v>
@@ -14420,10 +14420,10 @@
         <v>0.0442013196579361</v>
       </c>
       <c r="M275" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N275" t="n">
-        <v>0.128128470146066</v>
+        <v>0.0683351840779021</v>
       </c>
       <c r="O275" t="b">
         <v>0</v>
@@ -14470,10 +14470,10 @@
         <v>0.02516111023792</v>
       </c>
       <c r="M276" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="N276" t="n">
-        <v>0.104602510460251</v>
+        <v>0.0643707756678468</v>
       </c>
       <c r="O276" t="b">
         <v>0</v>
@@ -14870,10 +14870,10 @@
         <v>0.0312896121744421</v>
       </c>
       <c r="M284" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N284" t="n">
-        <v>0.123690937577307</v>
+        <v>0.0659685000412303</v>
       </c>
       <c r="O284" t="b">
         <v>0</v>
@@ -15020,10 +15020,10 @@
         <v>0.0352662913381714</v>
       </c>
       <c r="M287" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="N287" t="n">
-        <v>0.118422026496928</v>
+        <v>0.0666123899045222</v>
       </c>
       <c r="O287" t="b">
         <v>0</v>
@@ -15070,10 +15070,10 @@
         <v>0.0420348170760134</v>
       </c>
       <c r="M288" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="N288" t="n">
-        <v>0.105613778536031</v>
+        <v>0.0649930944837111</v>
       </c>
       <c r="O288" t="b">
         <v>0</v>
@@ -15220,10 +15220,10 @@
         <v>0.0366602215738631</v>
       </c>
       <c r="M291" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="N291" t="n">
-        <v>0.106356868199296</v>
+        <v>0.0654503804303363</v>
       </c>
       <c r="O291" t="b">
         <v>0</v>
@@ -15320,10 +15320,10 @@
         <v>0.0282236923226029</v>
       </c>
       <c r="M293" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N293" t="n">
-        <v>0.119980803071509</v>
+        <v>0.0639897616381379</v>
       </c>
       <c r="O293" t="b">
         <v>0</v>
@@ -15370,10 +15370,10 @@
         <v>0.0114347000556112</v>
       </c>
       <c r="M294" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="N294" t="n">
-        <v>0.101996211569285</v>
+        <v>0.0655689931516829</v>
       </c>
       <c r="O294" t="b">
         <v>0</v>
@@ -15470,10 +15470,10 @@
         <v>0.0723854955259819</v>
       </c>
       <c r="M296" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N296" t="n">
-        <v>0.124409056979348</v>
+        <v>0.0663514970556523</v>
       </c>
       <c r="O296" t="b">
         <v>0</v>
@@ -15620,10 +15620,10 @@
         <v>0.0556467609877703</v>
       </c>
       <c r="M299" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="N299" t="n">
-        <v>0.119751515605119</v>
+        <v>0.0673602275278797</v>
       </c>
       <c r="O299" t="b">
         <v>0</v>
@@ -15670,10 +15670,10 @@
         <v>0.0231906518093525</v>
       </c>
       <c r="M300" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="N300" t="n">
-        <v>0.103450823911919</v>
+        <v>0.0665041010862337</v>
       </c>
       <c r="O300" t="b">
         <v>0</v>
@@ -15770,10 +15770,10 @@
         <v>0.0515802787637369</v>
       </c>
       <c r="M302" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="N302" t="n">
-        <v>0.121645252033757</v>
+        <v>0.0684254542689881</v>
       </c>
       <c r="O302" t="b">
         <v>0</v>
@@ -15820,10 +15820,10 @@
         <v>0.0416781170232105</v>
       </c>
       <c r="M303" t="n">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="N303" t="n">
-        <v>0.103757503890906</v>
+        <v>0.066701252501297</v>
       </c>
       <c r="O303" t="b">
         <v>0</v>
@@ -15970,10 +15970,10 @@
         <v>0.0370378102646554</v>
       </c>
       <c r="M306" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N306" t="n">
-        <v>0.103610424802742</v>
+        <v>0.0717302940942058</v>
       </c>
       <c r="O306" t="b">
         <v>0</v>
@@ -16420,10 +16420,10 @@
         <v>0.0705123253394389</v>
       </c>
       <c r="M315" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="N315" t="n">
-        <v>0.103626943005181</v>
+        <v>0.0956556396970905</v>
       </c>
       <c r="O315" t="b">
         <v>0</v>
@@ -18770,10 +18770,10 @@
         <v>0.0430586168578055</v>
       </c>
       <c r="M362" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="N362" t="n">
-        <v>0.126606934164394</v>
+        <v>0.175301908843007</v>
       </c>
       <c r="O362" t="b">
         <v>0</v>
@@ -18820,10 +18820,10 @@
         <v>0.0389218766135965</v>
       </c>
       <c r="M363" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="N363" t="n">
-        <v>0.105160977188157</v>
+        <v>0.161786118751011</v>
       </c>
       <c r="O363" t="b">
         <v>0</v>
@@ -18920,10 +18920,10 @@
         <v>0.054462695541228</v>
       </c>
       <c r="M365" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="N365" t="n">
-        <v>0.120792398131744</v>
+        <v>0.169109357384442</v>
       </c>
       <c r="O365" t="b">
         <v>0</v>
@@ -18970,10 +18970,10 @@
         <v>0.0469420772746819</v>
       </c>
       <c r="M366" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="N366" t="n">
-        <v>0.106522451655195</v>
+        <v>0.155686660111439</v>
       </c>
       <c r="O366" t="b">
         <v>0</v>
@@ -19070,10 +19070,10 @@
         <v>0.0565582706433835</v>
       </c>
       <c r="M368" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="N368" t="n">
-        <v>0.126054494327548</v>
+        <v>0.174536992145835</v>
       </c>
       <c r="O368" t="b">
         <v>0</v>
@@ -19120,10 +19120,10 @@
         <v>0.0476175038836019</v>
       </c>
       <c r="M369" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="N369" t="n">
-        <v>0.0989690721649484</v>
+        <v>0.156701030927835</v>
       </c>
       <c r="O369" t="b">
         <v>0</v>
@@ -19220,10 +19220,10 @@
         <v>0.0563735440157395</v>
       </c>
       <c r="M371" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="N371" t="n">
-        <v>0.120163422254266</v>
+        <v>0.176239685972923</v>
       </c>
       <c r="O371" t="b">
         <v>0</v>
@@ -19270,10 +19270,10 @@
         <v>0.0403137701892689</v>
       </c>
       <c r="M372" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="N372" t="n">
-        <v>0.100893629287979</v>
+        <v>0.158547131738253</v>
       </c>
       <c r="O372" t="b">
         <v>0</v>
@@ -19370,10 +19370,10 @@
         <v>0.0574015638089767</v>
       </c>
       <c r="M374" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="N374" t="n">
-        <v>0.12421331566744</v>
+        <v>0.173898641934415</v>
       </c>
       <c r="O374" t="b">
         <v>0</v>
@@ -19420,10 +19420,10 @@
         <v>0.0434376834193166</v>
       </c>
       <c r="M375" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="N375" t="n">
-        <v>0.104175709697022</v>
+        <v>0.164944873686952</v>
       </c>
       <c r="O375" t="b">
         <v>0</v>
@@ -19520,10 +19520,10 @@
         <v>0.0712938227114923</v>
       </c>
       <c r="M377" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="N377" t="n">
-        <v>0.125659713495853</v>
+        <v>0.175923598894195</v>
       </c>
       <c r="O377" t="b">
         <v>0</v>
@@ -19570,10 +19570,10 @@
         <v>0.0465209592419369</v>
       </c>
       <c r="M378" t="n">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="N378" t="n">
-        <v>0.108774474256708</v>
+        <v>0.169204737732657</v>
       </c>
       <c r="O378" t="b">
         <v>0</v>
@@ -19670,10 +19670,10 @@
         <v>0.0932002144417741</v>
       </c>
       <c r="M380" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N380" t="n">
-        <v>0.120753501851554</v>
+        <v>0.064401867654162</v>
       </c>
       <c r="O380" t="b">
         <v>0</v>
@@ -19720,13 +19720,13 @@
         <v>0.0450347114330441</v>
       </c>
       <c r="M381" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N381" t="n">
-        <v>0.101825017623561</v>
+        <v>0.0704942429701574</v>
       </c>
       <c r="O381" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P381" t="b">
         <v>0</v>
@@ -19970,10 +19970,10 @@
         <v>0.0633946848437411</v>
       </c>
       <c r="M386" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="N386" t="n">
-        <v>0.12100128563866</v>
+        <v>0.0680632231717462</v>
       </c>
       <c r="O386" t="b">
         <v>0</v>
@@ -20020,10 +20020,10 @@
         <v>0.0823908096815058</v>
       </c>
       <c r="M387" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N387" t="n">
-        <v>0.104300385109114</v>
+        <v>0.0722079589216945</v>
       </c>
       <c r="O387" t="b">
         <v>0</v>
@@ -20120,10 +20120,10 @@
         <v>0.0537437457968037</v>
       </c>
       <c r="M389" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N389" t="n">
-        <v>0.12347711557458</v>
+        <v>0.0658544616397761</v>
       </c>
       <c r="O389" t="b">
         <v>0</v>
@@ -20170,10 +20170,10 @@
         <v>0.0201077019473549</v>
       </c>
       <c r="M390" t="n">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="N390" t="n">
-        <v>0.106765019897117</v>
+        <v>0.0679413762981656</v>
       </c>
       <c r="O390" t="b">
         <v>0</v>
@@ -20270,10 +20270,10 @@
         <v>0.0441196797022246</v>
       </c>
       <c r="M392" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N392" t="n">
-        <v>0.126230749810654</v>
+        <v>0.0673230665656821</v>
       </c>
       <c r="O392" t="b">
         <v>0</v>
@@ -20320,10 +20320,10 @@
         <v>0.0163621468962998</v>
       </c>
       <c r="M393" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N393" t="n">
-        <v>0.0988467874794069</v>
+        <v>0.0658978583196046</v>
       </c>
       <c r="O393" t="b">
         <v>0</v>
@@ -20570,10 +20570,10 @@
         <v>0.0870756405949396</v>
       </c>
       <c r="M398" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="N398" t="n">
-        <v>0.121477162293489</v>
+        <v>0.170068027210884</v>
       </c>
       <c r="O398" t="b">
         <v>0</v>
@@ -20620,10 +20620,10 @@
         <v>0.0871697045874413</v>
       </c>
       <c r="M399" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="N399" t="n">
-        <v>0.108479479298499</v>
+        <v>0.162719218947749</v>
       </c>
       <c r="O399" t="b">
         <v>0</v>
@@ -20720,10 +20720,10 @@
         <v>0.0589846098359881</v>
       </c>
       <c r="M401" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="N401" t="n">
-        <v>0.128789379829602</v>
+        <v>0.178323756687141</v>
       </c>
       <c r="O401" t="b">
         <v>0</v>
@@ -20770,10 +20770,10 @@
         <v>0.0279766495171053</v>
       </c>
       <c r="M402" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="N402" t="n">
-        <v>0.0986941998177953</v>
+        <v>0.159429092013362</v>
       </c>
       <c r="O402" t="b">
         <v>0</v>
@@ -20870,10 +20870,10 @@
         <v>0.0501047152868525</v>
       </c>
       <c r="M404" t="n">
-        <v>15</v>
+        <v>22</v>
       </c>
       <c r="N404" t="n">
-        <v>0.120375571783966</v>
+        <v>0.176550838616483</v>
       </c>
       <c r="O404" t="b">
         <v>0</v>
@@ -20920,10 +20920,10 @@
         <v>0.0346669668364871</v>
       </c>
       <c r="M405" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="N405" t="n">
-        <v>0.100177236649457</v>
+        <v>0.161824766895276</v>
       </c>
       <c r="O405" t="b">
         <v>0</v>
@@ -21020,10 +21020,10 @@
         <v>0.047367602281753</v>
       </c>
       <c r="M407" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="N407" t="n">
-        <v>0.119967009072505</v>
+        <v>0.172452575541726</v>
       </c>
       <c r="O407" t="b">
         <v>0</v>
@@ -21070,10 +21070,10 @@
         <v>0.0940611559363081</v>
       </c>
       <c r="M408" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="N408" t="n">
-        <v>0.103355064398156</v>
+        <v>0.159007791381778</v>
       </c>
       <c r="O408" t="b">
         <v>0</v>
@@ -21170,10 +21170,10 @@
         <v>0.0566139855181378</v>
       </c>
       <c r="M410" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="N410" t="n">
-        <v>0.125763564498742</v>
+        <v>0.179662234998203</v>
       </c>
       <c r="O410" t="b">
         <v>0</v>
@@ -21220,10 +21220,10 @@
         <v>0.0908277658639352</v>
       </c>
       <c r="M411" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="N411" t="n">
-        <v>0.112828613336342</v>
+        <v>0.169242920004513</v>
       </c>
       <c r="O411" t="b">
         <v>0</v>
@@ -21470,10 +21470,10 @@
         <v>0.0474261277526193</v>
       </c>
       <c r="M416" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="N416" t="n">
-        <v>0.120804210889637</v>
+        <v>0.172577444128052</v>
       </c>
       <c r="O416" t="b">
         <v>0</v>
@@ -21520,10 +21520,10 @@
         <v>0.0718408536621055</v>
       </c>
       <c r="M417" t="n">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="N417" t="n">
-        <v>0.0988979937835547</v>
+        <v>0.155411133088443</v>
       </c>
       <c r="O417" t="b">
         <v>0</v>
@@ -21620,10 +21620,10 @@
         <v>0.127185674566487</v>
       </c>
       <c r="M419" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="N419" t="n">
-        <v>0.125920185974429</v>
+        <v>0.174351026733824</v>
       </c>
       <c r="O419" t="b">
         <v>0</v>
@@ -21670,10 +21670,10 @@
         <v>0.0594746595237704</v>
       </c>
       <c r="M420" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="N420" t="n">
-        <v>0.105064089094348</v>
+        <v>0.168102542550956</v>
       </c>
       <c r="O420" t="b">
         <v>0</v>
@@ -21770,10 +21770,10 @@
         <v>0.032636639322883</v>
       </c>
       <c r="M422" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="N422" t="n">
-        <v>0.122337363270006</v>
+        <v>0.172711571675302</v>
       </c>
       <c r="O422" t="b">
         <v>0</v>
@@ -21820,13 +21820,13 @@
         <v>0.133973038988039</v>
       </c>
       <c r="M423" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="N423" t="n">
-        <v>0.105374077976818</v>
+        <v>0.158061116965227</v>
       </c>
       <c r="O423" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P423" t="b">
         <v>0</v>
@@ -21970,10 +21970,10 @@
         <v>0.0318281718061333</v>
       </c>
       <c r="M426" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="N426" t="n">
-        <v>0.103404390709513</v>
+        <v>0.159083678014636</v>
       </c>
       <c r="O426" t="b">
         <v>0</v>
@@ -22070,10 +22070,10 @@
         <v>0.0548705102126687</v>
       </c>
       <c r="M428" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="N428" t="n">
-        <v>0.131737841695027</v>
+        <v>0.186628609067955</v>
       </c>
       <c r="O428" t="b">
         <v>0</v>
@@ -22370,10 +22370,10 @@
         <v>0.0216268712241299</v>
       </c>
       <c r="M434" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N434" t="n">
-        <v>0.121546065958998</v>
+        <v>0.0648245685114658</v>
       </c>
       <c r="O434" t="b">
         <v>0</v>
@@ -22520,10 +22520,10 @@
         <v>0.0677277285332524</v>
       </c>
       <c r="M437" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N437" t="n">
-        <v>0.121310149615851</v>
+        <v>0.0646987464617873</v>
       </c>
       <c r="O437" t="b">
         <v>0</v>
@@ -22570,10 +22570,10 @@
         <v>0.0105891572505972</v>
       </c>
       <c r="M438" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="N438" t="n">
-        <v>0.102774922918808</v>
+        <v>0.0711518697130208</v>
       </c>
       <c r="O438" t="b">
         <v>0</v>
@@ -22720,10 +22720,10 @@
         <v>0.0166824262105218</v>
       </c>
       <c r="M441" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
       <c r="N441" t="n">
-        <v>0.106382978723404</v>
+        <v>0.0654664484451719</v>
       </c>
       <c r="O441" t="b">
         <v>0</v>
@@ -22820,10 +22820,10 @@
         <v>0.0360420657677967</v>
       </c>
       <c r="M443" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="N443" t="n">
-        <v>0.125397090787494</v>
+        <v>0.0668784484199967</v>
       </c>
       <c r="O443" t="b">
         <v>0</v>
@@ -22870,10 +22870,10 @@
         <v>0.0343605227223589</v>
       </c>
       <c r="M444" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N444" t="n">
-        <v>0.108774474256708</v>
+        <v>0.0725163161711385</v>
       </c>
       <c r="O444" t="b">
         <v>0</v>
@@ -22970,10 +22970,10 @@
         <v>0.0437208424765784</v>
       </c>
       <c r="M446" t="n">
-        <v>13</v>
+        <v>7</v>
       </c>
       <c r="N446" t="n">
-        <v>0.123071097226167</v>
+        <v>0.0662690523525514</v>
       </c>
       <c r="O446" t="b">
         <v>0</v>
@@ -23020,13 +23020,13 @@
         <v>0.0610065456886325</v>
       </c>
       <c r="M447" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="N447" t="n">
-        <v>0.102660621096758</v>
+        <v>0.0684404140645051</v>
       </c>
       <c r="O447" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P447" t="b">
         <v>0</v>
@@ -23270,10 +23270,10 @@
         <v>0.0566385866157966</v>
       </c>
       <c r="M452" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="N452" t="n">
-        <v>0.125372198714935</v>
+        <v>0.172386773233036</v>
       </c>
       <c r="O452" t="b">
         <v>0</v>
@@ -23320,10 +23320,10 @@
         <v>0.0285559013965602</v>
       </c>
       <c r="M453" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="N453" t="n">
-        <v>0.104484809516155</v>
+        <v>0.160745860794085</v>
       </c>
       <c r="O453" t="b">
         <v>0</v>
@@ -23420,10 +23420,10 @@
         <v>0.046677766202464</v>
       </c>
       <c r="M455" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="N455" t="n">
-        <v>0.123375555189998</v>
+        <v>0.172725777265998</v>
       </c>
       <c r="O455" t="b">
         <v>0</v>
@@ -23470,10 +23470,10 @@
         <v>0.0296242465483012</v>
       </c>
       <c r="M456" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="N456" t="n">
-        <v>0.0980761976612599</v>
+        <v>0.15843078083742</v>
       </c>
       <c r="O456" t="b">
         <v>0</v>
@@ -23570,10 +23570,10 @@
         <v>0.0552722507744152</v>
       </c>
       <c r="M458" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="N458" t="n">
-        <v>0.120964693430105</v>
+        <v>0.173886746805776</v>
       </c>
       <c r="O458" t="b">
         <v>0</v>
@@ -23620,10 +23620,10 @@
         <v>0.03098848965064</v>
       </c>
       <c r="M459" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="N459" t="n">
-        <v>0.0988593155893536</v>
+        <v>0.159695817490494</v>
       </c>
       <c r="O459" t="b">
         <v>0</v>
@@ -23720,10 +23720,10 @@
         <v>0.0538908498045714</v>
       </c>
       <c r="M461" t="n">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="N461" t="n">
-        <v>0.119289874394779</v>
+        <v>0.168409234439688</v>
       </c>
       <c r="O461" t="b">
         <v>0</v>
@@ -23770,10 +23770,10 @@
         <v>0.0768061096222524</v>
       </c>
       <c r="M462" t="n">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="N462" t="n">
-        <v>0.104948736578671</v>
+        <v>0.161459594736417</v>
       </c>
       <c r="O462" t="b">
         <v>0</v>
@@ -23870,10 +23870,10 @@
         <v>0.0453301855996467</v>
       </c>
       <c r="M464" t="n">
-        <v>15</v>
+        <v>21</v>
       </c>
       <c r="N464" t="n">
-        <v>0.125156445556946</v>
+        <v>0.175219023779725</v>
       </c>
       <c r="O464" t="b">
         <v>0</v>
@@ -23920,10 +23920,10 @@
         <v>0.0286634811152069</v>
       </c>
       <c r="M465" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="N465" t="n">
-        <v>0.110265740434447</v>
+        <v>0.165398610651671</v>
       </c>
       <c r="O465" t="b">
         <v>0</v>
@@ -24020,10 +24020,10 @@
         <v>0.0724926808580702</v>
       </c>
       <c r="M467" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="N467" t="n">
-        <v>0.126050420168067</v>
+        <v>0.178571428571429</v>
       </c>
       <c r="O467" t="b">
         <v>0</v>
@@ -24070,10 +24070,10 @@
         <v>0.0450646172100378</v>
       </c>
       <c r="M468" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="N468" t="n">
-        <v>0.115995824150331</v>
+        <v>0.173993736225496</v>
       </c>
       <c r="O468" t="b">
         <v>0</v>
@@ -25070,10 +25070,10 @@
         <v>0.110430069440483</v>
       </c>
       <c r="M488" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="N488" t="n">
-        <v>0.119415566170273</v>
+        <v>0.210733352065187</v>
       </c>
       <c r="O488" t="b">
         <v>0</v>
@@ -25220,10 +25220,10 @@
         <v>0.0389496885617358</v>
       </c>
       <c r="M491" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="N491" t="n">
-        <v>0.121367887484829</v>
+        <v>0.214178624973228</v>
       </c>
       <c r="O491" t="b">
         <v>0</v>
@@ -25370,10 +25370,10 @@
         <v>0.0509466415658861</v>
       </c>
       <c r="M494" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="N494" t="n">
-        <v>0.124542124542125</v>
+        <v>0.212454212454212</v>
       </c>
       <c r="O494" t="b">
         <v>0</v>
@@ -25520,10 +25520,10 @@
         <v>0.0746246846655437</v>
       </c>
       <c r="M497" t="n">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="N497" t="n">
-        <v>0.126752752911352</v>
+        <v>0.213895270537907</v>
       </c>
       <c r="O497" t="b">
         <v>0</v>
@@ -25670,10 +25670,10 @@
         <v>0.0477746421121876</v>
       </c>
       <c r="M500" t="n">
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="N500" t="n">
-        <v>0.119545726240287</v>
+        <v>0.212525735538288</v>
       </c>
       <c r="O500" t="b">
         <v>0</v>

</xml_diff>